<commit_message>
Pi/Display power board RC1.1: library footprints, 5V drop budget, DNP trim pads
Replace hand-drawn footprints with official KiCad ones (fixes Micro-Fit
row numbering and Nano2 size), re-lay the 5V path, add voltage-drop budget
script/doc, 16 AWG/150 mm harness, DNP trim network. RSDW40F-05 footprint is
still an unverified placeholder; RC2 intentionally not generated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ENatZXrEDA18PaxUrZWrpi
</commit_message>
<xml_diff>
--- a/OSBAMS_Pi_Display_Power_RevA_RC1/bom/OSBAMS_Pi_Display_Power_RevA_RC1_BOM.xlsx
+++ b/OSBAMS_Pi_Display_Power_RevA_RC1/bom/OSBAMS_Pi_Display_Power_RevA_RC1_BOM.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -525,7 +525,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>RSDW40_PLACEHOLDER</t>
+          <t>OSBAMS_PiPwr:RSDW40F-05_PLACEHOLDER_UNVERIFIED</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>FOOTPRINT PLACEHOLDER - verify vs Mean Well drawing</t>
+          <t>FOOTPRINT PLACEHOLDER - OPEN: verify vs Mean Well drawing</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>FUSE_NANO2_H</t>
+          <t>Fuse:Fuse_Littelfuse-NANO2-451_453</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Land pattern unverified</t>
+          <t>Footprint: official KiCad library (generated from manufacturer datasheet); NOT cross-checked against the manufacturer PDF</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>FUSE_NANO2_V</t>
+          <t>Fuse:Fuse_Littelfuse-NANO2-451_453</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Land pattern unverified</t>
+          <t>Footprint: official KiCad library (generated from manufacturer datasheet); NOT cross-checked against the manufacturer PDF</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>DO214AA</t>
+          <t>Diode_SMD:D_SMB</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>MPN from design brief/selection; stock + land pattern not verified offline</t>
+          <t>Footprint: official KiCad library (generated from manufacturer datasheet); NOT cross-checked against the manufacturer PDF</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>MICROFIT_RA_2</t>
+          <t>Connector_Molex:Molex_Micro-Fit_3.0_43045-0200_2x01_P3.00mm_Horizontal</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Footprint + mating parts unverified</t>
+          <t>Footprint: official KiCad library (generated from manufacturer datasheet); NOT cross-checked against the manufacturer PDF; mating parts unverified</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>MICROFIT_RA_4</t>
+          <t>Connector_Molex:Molex_Micro-Fit_3.0_43045-0400_2x02_P3.00mm_Horizontal</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Footprint + mating parts unverified</t>
+          <t>Footprint: official KiCad library (generated from manufacturer datasheet); NOT cross-checked against the manufacturer PDF (pegs + drills included); mating parts unverified</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>C0603</t>
+          <t>Capacitor_SMD:C_0603_1608Metric</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>CP_RADIAL_D8_P35</t>
+          <t>Capacitor_THT:CP_Radial_D8.0mm_P3.50mm</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Package/pitch unverified</t>
+          <t>Footprint: official KiCad library (generated from manufacturer datasheet); NOT cross-checked against the manufacturer PDF; verify body D8/pitch 3.5 vs EEU-FM1H101</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>CP_RADIAL_D10_P50</t>
+          <t>Capacitor_THT:CP_Radial_D10.0mm_P5.00mm</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Package/pitch unverified</t>
+          <t>Footprint: official KiCad library (generated from manufacturer datasheet); NOT cross-checked against the manufacturer PDF; verify body D10/pitch 5.0 vs EEU-FR1C681</t>
         </is>
       </c>
     </row>
@@ -975,7 +975,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>C0805</t>
+          <t>Capacitor_SMD:C_0805_2012Metric</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>LED0603</t>
+          <t>LED_SMD:LED_0603_1608Metric</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TP1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1105,27 +1105,27 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>12V_IN</t>
+          <t>DNP</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>SMT test point</t>
+          <t>TRIM option resistor TRIM-&gt;+VOUT. DO NOT FIT unless Mean Well trim formula confirmed (value TBD)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Keystone</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>5015</t>
+          <t>RC0603FR-07TBDL</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>TP15</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1135,19 +1135,19 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Confirm stock/lifecycle at order</t>
+          <t>DNP</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>MPN from design brief/selection; stock + land pattern not verified offline</t>
+          <t>DNP - do not fit</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TP2</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
@@ -1155,27 +1155,27 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>12V_GND</t>
+          <t>DNP</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>SMT test point</t>
+          <t>TRIM option resistor TRIM-&gt;-VOUT. DO NOT FIT unless Mean Well trim formula confirmed (value TBD)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Keystone</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>5015</t>
+          <t>RC0603FR-07TBDL</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>TP15</t>
+          <t>Resistor_SMD:R_0603_1608Metric</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1185,19 +1185,19 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Confirm stock/lifecycle at order</t>
+          <t>DNP</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>MPN from design brief/selection; stock + land pattern not verified offline</t>
+          <t>DNP - do not fit</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TP3</t>
+          <t>TP1</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>5V_ISO_RAW</t>
+          <t>12V_IN</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>TP15</t>
+          <t>TestPoint:TestPoint_Pad_D1.5mm</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TP4</t>
+          <t>TP2</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>5V_PI</t>
+          <t>12V_GND</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>TP15</t>
+          <t>TestPoint:TestPoint_Pad_D1.5mm</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1297,7 +1297,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TP5</t>
+          <t>TP3</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>PI_GND</t>
+          <t>5V_ISO_RAW</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>TP15</t>
+          <t>TestPoint:TestPoint_Pad_D1.5mm</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1345,130 +1345,146 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
-      <c r="J19" s="2" t="n"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TP4</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>5V_PI</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>SMT test point</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Keystone</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>5015</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>TestPoint:TestPoint_Pad_D1.5mm</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>SMD</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Confirm stock/lifecycle at order</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>MPN from design brief/selection; stock + land pattern not verified offline</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>MATING HARNESS PARTS (not on PCB) - all candidates, verify against Molex 43025/43030 and 214755 families</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
+          <t>TP5</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>PI_GND</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>SMT test point</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Keystone</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>5015</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>TestPoint:TestPoint_Pad_D1.5mm</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>SMD</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Confirm stock/lifecycle at order</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>MPN from design brief/selection; stock + land pattern not verified offline</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>J_OUT mate</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Micro-Fit 3.0 receptacle housing, 4 circuits, dual row</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Molex</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>43025-0400</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Harness</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>Keyed; mates J_OUT 430450400</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>J_IN mate</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Micro-Fit 3.0 receptacle housing, 2 circuits</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Molex</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>43025-0200</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>Harness</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>Keyed; mates J_IN 430450200</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
+          <t>MATING HARNESS PARTS (not on PCB) - all candidates, verify against Molex 43025/43030 and 214755 families</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Terminals</t>
+          <t>J_OUT mate</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Micro-Fit 3.0 crimp terminals (43030 family) - 4 out + 2 in, wire 18 AWG</t>
+          <t>Micro-Fit 3.0 receptacle housing, 4 circuits, dual row</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1478,7 +1494,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>43030-0007 (candidate)</t>
+          <t>43025-0400</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
@@ -1489,19 +1505,19 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Select exact terminal for 18 AWG insulation OD; confirm current rating</t>
+          <t>Keyed; mates J_OUT 430450400</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Verify - candidate only</t>
+          <t>Verify</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Pi-side housing</t>
+          <t>J_IN mate</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1510,17 +1526,17 @@
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2.54 mm pitch 2x5 crimp housing for Pi GPIO pins 1-10, populate cavities 2,4,6,9 only</t>
+          <t>Micro-Fit 3.0 receptacle housing, 2 circuits</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Molex</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>43025-0200</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
@@ -1531,38 +1547,38 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Choose crimp housing + terminals rated &gt;=3 A/contact; NO Dupont jumpers</t>
+          <t>Keyed; mates J_IN 430450200</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>Verify</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Wire</t>
+          <t>Terminals</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C25" s="2" t="inlineStr"/>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>18 AWG (or 16 AWG) stranded silicone, red/black, &lt;=250 mm</t>
+          <t>Micro-Fit 3.0 crimp terminals (43030 family) - 4 out + 2 in, wire 18 AWG</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Molex</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>43030-0007 (candidate)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
@@ -1571,8 +1587,92 @@
           <t>Harness</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Select exact terminal for 18 AWG insulation OD; confirm current rating</t>
+        </is>
+      </c>
       <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Verify - candidate only</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Pi-side housing</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>2.54 mm pitch 2x5 crimp housing for Pi GPIO pins 1-10, populate cavities 2,4,6,9 only</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Harness</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Choose crimp housing + terminals rated &gt;=3 A/contact; NO Dupont jumpers</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Wire</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>18 AWG (or 16 AWG) stranded silicone, red/black, &lt;=250 mm</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Harness</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>

</xml_diff>

<commit_message>
Budget at +-1% with Harwin M20 Pi end; exact trim-up Rt; Pi-end reversal hazard
Closes the voltage budget on paper (trim to 5.14 V, Rt 105k, R3 DNP).
Pi-end pin map/keying, RSDW pin XY, KiCad 10 ERC and bench remain open.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ENatZXrEDA18PaxUrZWrpi
</commit_message>
<xml_diff>
--- a/OSBAMS_Pi_Display_Power_RevA_RC1/bom/OSBAMS_Pi_Display_Power_RevA_RC1_BOM.xlsx
+++ b/OSBAMS_Pi_Display_Power_RevA_RC1/bom/OSBAMS_Pi_Display_Power_RevA_RC1_BOM.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1610,17 +1610,17 @@
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2.54 mm pitch 2x5 crimp housing for Pi GPIO pins 1-10, populate cavities 2,4,6,9 only</t>
+          <t>Harwin M20 2x5 cable housing, populate cavities 2,4,6,9 only (UNPOLARISED - needs anti-reversal key)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Harwin</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>M20-1070500</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
@@ -1631,38 +1631,38 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Choose crimp housing + terminals rated &gt;=3 A/contact; NO Dupont jumpers</t>
+          <t>Owner-cited; confirm layout on Harwin drawing</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>Owner-cited</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Wire</t>
+          <t>Pi-side contacts</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>18 AWG (or 16 AWG) stranded silicone, red/black, &lt;=250 mm</t>
+          <t>Harwin M20 gold crimp contact, 22-30 AWG, 3 A, 20 mOhm max</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Harwin</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>M20-1160042</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
@@ -1671,8 +1671,92 @@
           <t>Harness</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>22 AWG branch leads; 2x +5V, 2x GND</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Owner-cited</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Anti-reversal key / interposer</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Mechanical key or keyed interposer for Pi end</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Harness</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Reversed housing swaps +5V and GND - decision required</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Wire</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>16 AWG trunk (&lt;=150 mm) + 22 AWG branch leads (~50 mm), red/black</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Harness</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>

</xml_diff>

<commit_message>
Keyed Pi interposer, F1 8A time-delay, calibration procedure, budget update
Add OSBAMS_Pi_Power_Interposer_RevA_RC1 (Micro-Fit + 2x20 stacking socket, key
standoffs), trim calibration script/procedure/acceptance record, F1 candidate
0453008.MRL, budget with interposer path. RC2 still gated: F1 datasheet,
socket MPN, key 3D check, KiCad 10 ERC.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ENatZXrEDA18PaxUrZWrpi
</commit_message>
<xml_diff>
--- a/OSBAMS_Pi_Display_Power_RevA_RC1/bom/OSBAMS_Pi_Display_Power_RevA_RC1_BOM.xlsx
+++ b/OSBAMS_Pi_Display_Power_RevA_RC1/bom/OSBAMS_Pi_Display_Power_RevA_RC1_BOM.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -555,12 +555,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>5A 125V</t>
+          <t>8A 125V TD</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Nano2 SMD fuse, fast-acting, 5 A, 125 VAC/VDC (input)</t>
+          <t>Nano2 SMD fuse, TIME-DELAY (Slo-Blo class), 8 A (input) - per Mean Well input-fuse recommendation</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>0451005.MRL</t>
+          <t>0453008.MRL</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -585,12 +585,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Active; DigiKey-stocked per design brief</t>
+          <t>CANDIDATE - confirm exact 8 A time-delay MPN and stock CANDIDATE - datasheet (DC cold R, DC voltage, interrupt rating, I2t) not yet verified</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Footprint: official KiCad library (generated from manufacturer datasheet); NOT cross-checked against the manufacturer PDF</t>
+          <t>Footprint: official KiCad library (generated from manufacturer datasheet); NOT cross-checked against the manufacturer PDF; MPN is a CANDIDATE (8 A time-delay): verify DC R, DC voltage rating, interrupt rating, I2t</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Pi-side housing</t>
+          <t>Pi-end interposer</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1610,17 +1610,17 @@
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Harwin M20 2x5 cable housing, populate cavities 2,4,6,9 only (UNPOLARISED - needs anti-reversal key)</t>
+          <t>OSBAMS_Pi_Power_Interposer_RevA (keyed Micro-Fit to Pi GPIO) - see its own BOM</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Harwin</t>
+          <t>OSBAMS</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>M20-1070500</t>
+          <t>Interposer RevA RC1</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
@@ -1631,38 +1631,38 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Owner-cited; confirm layout on Harwin drawing</t>
+          <t>Replaces Harwin M20 housing</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Owner-cited</t>
+          <t>Designed; socket MPN + key 3D check open</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Pi-side contacts</t>
+          <t>Wire</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Harwin M20 gold crimp contact, 22-30 AWG, 3 A, 20 mOhm max</t>
+          <t>16 AWG, &lt;=150 mm, red/black, 4 wires, 1:1 to the interposer</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Harwin</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>M20-1160042</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
@@ -1671,92 +1671,8 @@
           <t>Harness</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>22 AWG branch leads; 2x +5V, 2x GND</t>
-        </is>
-      </c>
+      <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>Owner-cited</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Anti-reversal key / interposer</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Mechanical key or keyed interposer for Pi end</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>Harness</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>Reversed housing swaps +5V and GND - decision required</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Wire</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" s="2" t="inlineStr"/>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>16 AWG trunk (&lt;=150 mm) + 22 AWG branch leads (~50 mm), red/black</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>Harness</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>

</xml_diff>

<commit_message>
F1 -> Littelfuse 407 8A time-lag (0407008.WR); F2 verified; interposer to HAT+ geometry
Remove 0453008.MRL (very fast-acting). F1 datasheet values and 1206 land pattern
implemented; F2 footprint verified against 451/453 datasheet. Interposer now 65 mm
with M2.5 mounting holes per HAT+ spec. RC2 still gated: socket MPN, Pi 5 STEP
keying check, KiCad 10 ERC.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ENatZXrEDA18PaxUrZWrpi
</commit_message>
<xml_diff>
--- a/OSBAMS_Pi_Display_Power_RevA_RC1/bom/OSBAMS_Pi_Display_Power_RevA_RC1_BOM.xlsx
+++ b/OSBAMS_Pi_Display_Power_RevA_RC1/bom/OSBAMS_Pi_Display_Power_RevA_RC1_BOM.xlsx
@@ -525,7 +525,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>OSBAMS_PiPwr:RSDW40F-05_PLACEHOLDER_UNVERIFIED</t>
+          <t>OSBAMS_PiPwr:RSDW40F-05_MeanWell_2x1in</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -555,12 +555,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>8A 125V TD</t>
+          <t>8A TIME-LAG 24V</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Nano2 SMD fuse, TIME-DELAY (Slo-Blo class), 8 A (input) - per Mean Well input-fuse recommendation</t>
+          <t>407 Series 1206 time-lag SMD fuse, 8 A, 24 V max, 60 A@24VDC interrupt (input; Mean Well recommends 8 A delay type)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -570,12 +570,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>0453008.MRL</t>
+          <t>0407008.WR</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Fuse:Fuse_Littelfuse-NANO2-451_453</t>
+          <t>OSBAMS_PiPwr:Fuse_1206_Littelfuse407</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -585,12 +585,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>CANDIDATE - confirm exact 8 A time-delay MPN and stock CANDIDATE - datasheet (DC cold R, DC voltage, interrupt rating, I2t) not yet verified</t>
+          <t>Confirm PCBWay/DigiKey stock for 0407008.WR (reel 3000; ask for cut tape/qty) Datasheet-verified: 9 mOhm nominal, I2t 24.12 A2s, 0.097 V drop @8 A</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Footprint: official KiCad library (generated from manufacturer datasheet); NOT cross-checked against the manufacturer PDF; MPN is a CANDIDATE (8 A time-delay): verify DC R, DC voltage rating, interrupt rating, I2t</t>
+          <t>Datasheet-verified (Littelfuse 407, rev 09/14/20): 8 A time-lag, 24 V, 60 A@24VDC, 9 mOhm, I2t 24.12; land pattern = datasheet recommended pads</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Footprint: official KiCad library (generated from manufacturer datasheet); NOT cross-checked against the manufacturer PDF</t>
+          <t>Datasheet-verified (451/453 rev): 8 A very fast-acting, 125 V, 7.7 mOhm cold, I2t 20.23; pads 1.96x3.15, span 6.86 match the library footprint</t>
         </is>
       </c>
     </row>

</xml_diff>